<commit_message>
Store 4P Index score columns as numeric types in xlsx (not text)
Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/4p-index/STP_Decreto-36-1999_Waste-Decree_4P-Index.xlsx
+++ b/4p-index/STP_Decreto-36-1999_Waste-Decree_4P-Index.xlsx
@@ -588,61 +588,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E2" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G2" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I2" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K2" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="O2" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
@@ -654,25 +640,19 @@
           <t>Art. 1.º ('Princípio'): 'O detentor de resíduos sólidos, qualquer que seja a sua natureza e origem, deve promover a sua recolha, armazenagem, transporte e eliminação ou utilização, de tal forma que não ponham em perigo as espécies nem causem prejuízo ao ambiente.' / 'The holder of solid waste, whatever its nature and origin, must ensure its collection, storage, transport and disposal or use, in such a way that it does not endanger species or cause harm to the environment.'</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="S2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" s="2" t="n">
+        <v>0.5</v>
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Enforcement: Art. 34.º makes 'a prática de actos e actividades contrárias ao disposto no presente diploma' / 'the commission of acts and activities contrary to the provisions of this decree' an infraction subject to the sanctions process of Arts. 35.º–37.º (+0.25). No authority is specifically named within Art. 1.º itself (0). No monitoring mechanism specified within this article (0). Unconditional: the duty applies to any waste holder regardless of origin, with no exemption stated (+0.25).</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="V2" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
@@ -701,61 +681,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E3" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G3" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I3" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K3" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M3" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>0.69</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
+      <c r="O3" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>0.2</v>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
@@ -767,25 +733,19 @@
           <t>Art. 9.º(1): 'As Câmaras Distritais, as empresas e as unidades de saúde... devem organizar e manter actualizado um inventário que indique... as quantidades, natureza, origem e destino dos resíduos produzidos ou recolhidos, conforme o modelo constante do Anexo II.' / 'District Chambers, companies and health units... must organise and keep up to date an inventory indicating... the quantities, nature, origin and destination of the waste produced or collected, in accordance with the model set out in Annex II.' Annex II ('Mapa de Resíduos Sólidos' / 'Solid Waste Report') explicitly requires reporting of the average annual physical composition of collected waste by component, including 'Plástico' (Plastic) alongside metals, paper, glass, textiles, cardboard and fermentable materials, and separately requires reporting of quantities of recycled materials, again itemising 'Plástico' alongside paper, glass and metals. Art. 9.º(2): stricter registration requirements (storage, location and disposal conditions/methods) apply to toxic or hazardous waste. Art. 9.º(3): inventories and their data must be made available to entities with supervisory competence whenever requested.</t>
         </is>
       </c>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="S3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
           <t>Authority: District Chambers, companies and health units are explicitly designated as duty-bearers (+0.25). Monitoring: the inventory/reporting obligation is itself a data-collection mechanism, reinforced by Art. 9.º(3)'s requirement to make data available to supervisory entities on request (+0.25). Enforcement: not specifically tied within Art. 9.º itself (0). Unconditional: the general obligation applies without a stated exemption (hazardous waste is subject to additional, not fewer, requirements) (+0.25).</t>
         </is>
       </c>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>0.475</t>
-        </is>
+      <c r="V3" s="2" t="n">
+        <v>0.475</v>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
@@ -814,61 +774,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E4" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G4" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I4" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K4" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M4" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="O4" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
@@ -880,25 +826,19 @@
           <t>Art. 10.º ('Destino'): 'O destino a dar pelas empresas aos resíduos deve constar do processo de licenciamento, devendo ser indicada a previsão da natureza e da quantidade dos resíduos produzidos.' / 'The destination to be given by companies to their waste must be included in the licensing process, with an indication of the expected nature and quantity of the waste produced.' Art. 14.º: companies and health units are responsible for giving proper destination to their own waste under the terms of this decree, but may associate with District Chambers for collection, treatment, transport, storage, disposal or use, or with duly authorised consortia, where they lack their own means in the area where the waste is generated.</t>
         </is>
       </c>
-      <c r="S4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T4" s="2" t="inlineStr">
-        <is>
-          <t>0.25</t>
-        </is>
+      <c r="S4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>0.25</v>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
           <t>Enforcement: Art. 34.º general infractions clause covers breach of this obligation (+0.25). No specific authority named beyond the general licensing body (0). No monitoring mechanism specified within these articles (0). Not unconditional: Art. 14.º provides an alternative compliance route (association with District Chambers/authorised consortia) rather than a single unconditional obligation (0).</t>
         </is>
       </c>
-      <c r="V4" s="2" t="inlineStr">
-        <is>
-          <t>0.625</t>
-        </is>
+      <c r="V4" s="2" t="n">
+        <v>0.625</v>
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
@@ -927,61 +867,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E5" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G5" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I5" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K5" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M5" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="O5" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
@@ -993,25 +919,19 @@
           <t>Art. 11.º ('Recuperação'): 'Os projectos relativos à recuperação de resíduos, bem como os projectos de aproveitamento energético, são aprovados pelo membro do Governo responsável pelo sector do ambiente, que dará assistência técnica e tecnológica nos referidos projectos.' / 'Projects relating to the recovery of waste, as well as energy-recovery projects, are approved by the member of the Government responsible for the environment sector, who shall provide technical and technological assistance to such projects.'</t>
         </is>
       </c>
-      <c r="S5" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T5" s="2" t="inlineStr">
-        <is>
-          <t>0.25</t>
-        </is>
+      <c r="S5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>0.25</v>
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
           <t>Authority: the Government member responsible for the environment sector is explicitly designated as the approving authority (+0.25). No enforcement penalty specified (0). No monitoring mechanism specified (0). Not unconditional: approval is inherently a discretionary gatekeeping decision (0).</t>
         </is>
       </c>
-      <c r="V5" s="2" t="inlineStr">
-        <is>
-          <t>0.625</t>
-        </is>
+      <c r="V5" s="2" t="n">
+        <v>0.625</v>
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
@@ -1040,61 +960,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E6" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G6" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I6" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K6" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M6" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>0.69</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
+      <c r="O6" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>0.2</v>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
@@ -1106,25 +1012,19 @@
           <t>Art. 12.º(2): it is specifically incumbent upon the ministry responsible for the environment, having consulted the ministers of health, industry, commerce and tourism, to: (a) define national waste policy; (b) establish national and regional plans and general directives for the removal, treatment and final destination of waste; (c) issue binding opinions on projects submitted by District Chambers, individually or in association; and (d) make investments in sanitary landfills and other waste treatment and final-destination facilities. Art. 12.º(1): the licensing ministries and the environment ministry shall jointly regulate compliance specifications, including supervision and penalty conditions.</t>
         </is>
       </c>
-      <c r="S6" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T6" s="2" t="inlineStr">
-        <is>
-          <t>0.25</t>
-        </is>
+      <c r="S6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>0.25</v>
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
           <t>Authority: the environment ministry and other named ministries are explicitly designated (+0.25). No enforcement penalty specified within this article for the ministries' own non-performance (0). No monitoring mechanism specified (0). Not unconditional: these are policy-setting and planning functions, inherently discretionary in execution (0).</t>
         </is>
       </c>
-      <c r="V6" s="2" t="inlineStr">
-        <is>
-          <t>0.225</t>
-        </is>
+      <c r="V6" s="2" t="n">
+        <v>0.225</v>
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
@@ -1153,61 +1053,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E7" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G7" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I7" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K7" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M7" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>0.69</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
+      <c r="O7" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>0.2</v>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
@@ -1219,25 +1105,19 @@
           <t>Art. 13.º: without prejudice to Art. 9.º, District Chambers ('Câmaras Distritais'), within their areas of jurisdiction, are empowered to issue regulations adapted to their local specificities, with the objective of ensuring effective supervision and penalty enforcement under this decree, being responsible in particular for: (a) defining systems for the removal, treatment and final destination of waste produced within their jurisdiction and submitting the relevant projects for the opinion of the environment ministry; (b) promoting implementation of projects that received a favourable opinion and making the necessary investments; (c) publishing by-laws on waste collection and transport, setting out general guidelines for removal-plan operations; (d) planning, organising and promoting the collection, transport, disposal or use of waste; (e) ensuring the creation of sanitary landfills within their jurisdiction; and (f) collecting fines arising from infractions of this decree.</t>
         </is>
       </c>
-      <c r="S7" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T7" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="S7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
           <t>Authority: District Chambers are explicitly designated as the competent sub-national body (+0.25). Enforcement: Art. 13.º(f) explicitly empowers District Chambers to collect fines for infractions of the decree (+0.25). No monitoring mechanism specified within this article itself (0). Unconditional: no exemptions are stated to these competencies (+0.25).</t>
         </is>
       </c>
-      <c r="V7" s="2" t="inlineStr">
-        <is>
-          <t>0.475</t>
-        </is>
+      <c r="V7" s="2" t="n">
+        <v>0.475</v>
       </c>
       <c r="W7" s="2" t="inlineStr">
         <is>
@@ -1266,61 +1146,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E8" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G8" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I8" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K8" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M8" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="O8" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
@@ -1332,25 +1198,19 @@
           <t>Arts. 15.º–16.º: waste collection must be carried out using appropriate closed/covered receptacles suited to the type of waste, to be emptied with a frequency compatible with public health and hygiene requirements, particularly in urban areas. Art. 17.º: waste transport must, as a rule, be carried out in closed-body vehicles or vehicles fitted with appropriate covering devices; where a closed-body vehicle cannot be used, waste may be transported in open-body vehicles provided minimum health and safety standards are observed; this exception does not apply to the transport of hospital waste or toxic/hazardous waste. Art. 18.º ('Triagem'/Sorting): sorting consists of separating waste according to its nature, resulting in the separation of organic and inorganic matter.</t>
         </is>
       </c>
-      <c r="S8" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T8" s="2" t="inlineStr">
-        <is>
-          <t>0.25</t>
-        </is>
+      <c r="S8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" s="2" t="n">
+        <v>0.25</v>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
           <t>Enforcement: Art. 34.º general infractions clause covers breach of these standards (+0.25). No specific authority named within these articles (0). No monitoring mechanism specified (0). Not unconditional: Art. 17.º explicitly carves out hospital and toxic/hazardous waste from the open-body-vehicle exception, and more generally imposes differentiated standards by waste type (0).</t>
         </is>
       </c>
-      <c r="V8" s="2" t="inlineStr">
-        <is>
-          <t>0.625</t>
-        </is>
+      <c r="V8" s="2" t="n">
+        <v>0.625</v>
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
@@ -1379,61 +1239,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E9" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G9" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I9" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K9" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M9" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="O9" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
@@ -1445,25 +1291,19 @@
           <t>Art. 19.º(1): for the purposes of waste elimination and treatment, the following forms may be used: (a) sanitary landfill; (b) incineration; (c) composting; (d) recycling ('Reciclagem'). Art. 19.º(2)–(3): the siting rules of Art. 26.º apply equally to landfills, incineration and composting facilities. Art. 20.º: final destination should preferably be preceded by incineration or composting processes; in the case of sanitary landfill, the landfill itself is the final destination.</t>
         </is>
       </c>
-      <c r="S9" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T9" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="S9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>0.5</v>
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
           <t>Enforcement: Art. 34.º general infractions clause applies to use of non-listed/unlawful methods (+0.25). No authority specifically named within this article (0). No monitoring mechanism specified (0). Unconditional: the list of lawful methods (including recycling) is stated without exemption (+0.25).</t>
         </is>
       </c>
-      <c r="V9" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="V9" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
@@ -1492,61 +1332,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E10" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G10" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I10" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K10" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M10" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="O10" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
@@ -1558,25 +1384,19 @@
           <t>Art. 21.º ('Processos proibidos'): the following waste-disposal processes are prohibited within the territory of the Democratic Republic of São Tomé and Príncipe: (a) discharge into rivers, watercourses, the coastline, or in general at any point of national territory, without prior authorisation and outside sites designated for that purpose under this decree; (b) incineration at the locations referred to in the preceding point.</t>
         </is>
       </c>
-      <c r="S10" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T10" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="S10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T10" s="2" t="n">
+        <v>0.5</v>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
           <t>Enforcement: Art. 34.º general infractions clause applies (+0.25). No authority specifically named within this article (0). No monitoring mechanism specified (0). Unconditional: the prohibition is stated as a blanket ban with no exemption (+0.25).</t>
         </is>
       </c>
-      <c r="V10" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="V10" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="W10" s="2" t="inlineStr">
         <is>
@@ -1605,61 +1425,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E11" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G11" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I11" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K11" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M11" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="O11" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
@@ -1671,25 +1477,19 @@
           <t>Art. 22.º: sites intended for the treatment and final destination of waste are treated as industrial establishments and are therefore subject to licensing by the competent administrative body. Art. 23.º: the licensing file must address the admissible waste categories/types/quantities, identification/control/registration procedures, the processes/technologies used, and industrial-accident safety procedures. Art. 24.º: minimum technical requirements are set for each specific process — sanitary landfills (geological/hydrogeological characterisation, impact studies, operating methods, controls, post-closure use), incineration plants (incinerator type/capacity, temperature/residence time, flow and control systems, effluent characterisation, stack height), and physico-chemical treatment plants (methods used, contaminants removed, sludge/effluent characterisation and control); further procedures are left to future dedicated regulation (Art. 24.º(2)). Arts. 25.º–26.º: sanitary landfills must be sited more than 500 m from residential areas, agro-pastoral development areas, protected areas, water sources, riverbanks and the coastline, and no less than 200 m from the platform of national or secondary roads.</t>
         </is>
       </c>
-      <c r="S11" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T11" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="S11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>0.5</v>
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
           <t>Authority: the 'competente órgão da administração' / 'competent administrative body' is explicitly designated as the licensing authority (+0.25). Enforcement: Art. 34.º general infractions clause, plus licensing itself is a precondition for lawful operation (+0.25). No monitoring mechanism specified within these articles (0). Not unconditional: detailed procedures for each specific process are explicitly deferred to a future dedicated regulation (Art. 24.º(2)) (0).</t>
         </is>
       </c>
-      <c r="V11" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="V11" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="W11" s="2" t="inlineStr">
         <is>
@@ -1718,61 +1518,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E12" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G12" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I12" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K12" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M12" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>0.77</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
+      <c r="O12" s="2" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>0.6</v>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
@@ -1784,25 +1570,19 @@
           <t>Art. 27.º: without prejudice to the duties arising from the general polluter-pays principle already established under the Basic Environmental Law, benefits shall be encouraged and granted, under the framework the law shall establish, for investment in industrial activities for environmental conservation. Art. 28.º: the preceding paragraph shall apply to industrial units investing in: (a) priority recovery of toxic or hazardous waste; (b) reuse and/or recycling of waste, where recognised as the best techno-economic solution; (c) recovery of raw materials or energy production; (d) qualitative and quantitative reduction of the most harmful waste generated by the manufacturing industry.</t>
         </is>
       </c>
-      <c r="S12" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T12" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
           <t>Enabling power, not yet in force: Art. 27.º explicitly conditions the benefits on 'o quadro que a lei instituir' / 'the framework the law shall establish' — i.e., a future law not yet identified in this text — so no authority, enforcement or monitoring mechanism is evidenced, and the incentive is explicitly conditional on that future framework (0 on all four sub-scores).</t>
         </is>
       </c>
-      <c r="V12" s="2" t="inlineStr">
-        <is>
-          <t>0.3</t>
-        </is>
+      <c r="V12" s="2" t="n">
+        <v>0.3</v>
       </c>
       <c r="W12" s="2" t="inlineStr">
         <is>
@@ -1831,61 +1611,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E13" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G13" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I13" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K13" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M13" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>0.69</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
+      <c r="O13" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>0.2</v>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
@@ -1897,25 +1663,19 @@
           <t>Art. 29.º: the Supervision Council ('Conselho de Fiscalização', CF) is a control body charged with overseeing scrupulous compliance with this decree. Art. 30.º: the CF is composed of a president jointly appointed by the ministers responsible for the environment, health and industry, one member for each District Chamber in the country, and a civil-society representative drawn from environmental NGOs; the President has a casting vote. Art. 31.º: the CF is competent to: (a) carry out supervisory actions nationwide, at every stage of the waste-treatment process; (b) propose protection/conservation standards to the environment, health and industry ministries; (c) propose the creation of treatment stations to District Chambers; (d) issue inspection certificates for treatment stations and depots; and (e) ensure harmonisation of domestic law with relevant international conventions. Art. 32.º: the CF submits an annual activity report to the ministers of environment, health and industry. Art. 40.º: until the CF is created, the environment ministry shall exercise the functions assigned to it under this decree.</t>
         </is>
       </c>
-      <c r="S13" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T13" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="S13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>0.5</v>
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
           <t>Authority: the CF (and, as fallback under Art. 40.º, the environment ministry) is explicitly designated, with composition set out in Art. 30.º (+0.25). Monitoring: Art. 31.º(a) mandates nationwide supervisory action at every stage of the waste-treatment process (+0.25). Enforcement: the CF's own powers are inspection, certification and standard-proposal powers, not sanctioning powers (the sanctions regime is a separate instrument, Row 13) (0). Not unconditional: the CF's practical operation depends on it being formally constituted, notwithstanding the Art. 40.º ministerial fallback (0).</t>
         </is>
       </c>
-      <c r="V13" s="2" t="inlineStr">
-        <is>
-          <t>0.35</t>
-        </is>
+      <c r="V13" s="2" t="n">
+        <v>0.35</v>
       </c>
       <c r="W13" s="2" t="inlineStr">
         <is>
@@ -1944,61 +1704,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E14" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G14" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I14" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K14" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M14" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="O14" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
@@ -2010,25 +1756,19 @@
           <t>Art. 34.º: any act or activity contrary to the provisions of this decree constitutes an infraction. Art. 35.º: the sanctions process comprises citation followed by notification of the offender for voluntary payment of the fine; if voluntary payment is not made, the case is forwarded to the competent authorities for coercive collection; an offender caught in the act may be detained and handed over, together with the case file, to the competent authorities. Art. 36.º: fines range from Db 200,000 to 5,000,000 for individuals and from Db 500,000 to 10,000,000 for legal entities, depending on the gravity of the harmful act or conscious omission; attempt and negligence are punishable. Art. 37.º: accessory sanctions — where the gravity of the infraction so justifies — may include seizure of objects used as instruments of the infraction, loss of the right to subsidies granted by public entities or services, and suspension of the activity for up to two years.</t>
         </is>
       </c>
-      <c r="S14" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T14" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="S14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>0.5</v>
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
           <t>Authority: competent authorities receive the case file for coercive collection where voluntary payment fails (Art. 35.º(2)) (+0.25). Enforcement: this is itself the core sanctions/penalty regime, with fixed fine ranges and accessory sanctions (+0.25). No dedicated monitoring mechanism specified within these articles (relies on the CF/District Chambers, coded separately) (0). Not unconditional: accessory sanctions are explicitly discretionary and scaled to the gravity of the offence ('pode-se aplicar... quando a gravidade da infracção o justifique') (0).</t>
         </is>
       </c>
-      <c r="V14" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="V14" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="W14" s="2" t="inlineStr">
         <is>
@@ -2057,61 +1797,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E15" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G15" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I15" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K15" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M15" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>0.85</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="O15" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
@@ -2123,25 +1849,19 @@
           <t>Art. 38.º: independently of the sanctions to which agents are subject for infractions committed under this decree, and with a view to repairing damage caused to the environment, the administration may bring a civil indemnity action for losses and damages, seeking restitution and/or restoration of the affected area, in cases where this is possible.</t>
         </is>
       </c>
-      <c r="S15" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T15" s="2" t="inlineStr">
-        <is>
-          <t>0.25</t>
-        </is>
+      <c r="S15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="2" t="n">
+        <v>0.25</v>
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
           <t>Authority: 'a administração' / 'the administration' is explicitly designated as the holder of this power (+0.25). No automatic enforcement — the power is discretionary ('pode... intentar'), so not scored as enforcement (0). No monitoring mechanism specified (0). Not unconditional: explicitly limited to cases 'em que for possível' / 'where it is possible' (0).</t>
         </is>
       </c>
-      <c r="V15" s="2" t="inlineStr">
-        <is>
-          <t>0.625</t>
-        </is>
+      <c r="V15" s="2" t="n">
+        <v>0.625</v>
       </c>
       <c r="W15" s="2" t="inlineStr">
         <is>
@@ -2170,61 +1890,47 @@
           <t>Adopts the legal framework for the deposition, collection, transport, sorting and final disposal of municipal solid waste across national territory, with the explicit aim of encouraging lower solid-waste generation, developing recycling technologies, and ensuring that non-recycled waste is eliminated with maximum energy recovery, together with adequate environmental protection (Preamble). It contains an explicit, itemised reference to 'Plástico' (plastic) as a distinct waste-composition and recycled-material category in the mandatory Annex II waste-reporting template ('Mapa de Resíduos Sólidos') — the clearest explicit plastics reference identified so far in the São Tomé and Príncipe policy family. The decree assigns core implementation responsibility to District Chambers ('Câmaras Distritais')/municipal authorities (Art. 13), forming the base sub-national waste-management regime later updated by PAGIRSU/PNGIRSU.</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="E16" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="G16" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Executive decree ('Decreto') approved by the Council of Ministers — 'Visto e aprovado em Conselho de Ministros em S. Tomé, aos 25 de Fevereiro de 1999' / 'Seen and approved by the Council of Ministers in São Tomé, on 25 February 1999' — and promulgated by the President of the Republic on 3 August 1999, issued under Article 99(c) of the Constitution. Same Council of Ministers, signatories and promulgation date as the companion EIA Decree (37/1999); a sub-legislative executive instrument, not an Act passed by the National Assembly.</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="I16" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
           <t>waste management, municipalities, public health, industry, commerce/hospitality, agriculture</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
+      <c r="K16" s="2" t="n">
+        <v>0.75</v>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
           <t>production, recycling, disposal, environmental leakage</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="M16" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
           <t>Art. 39.º(1): 'As verbas arrecadadas das multas aplicadas aos infractores revertem-se a favor da câmara distrital com jurisdição sobre a área em que se registou a infracção, do agente ou grupo de agentes que a aplicaram, sob forma de emolumento, bem como a favor do Fundo para o Ambiente, a que se refere a Lei das Bases do Ambiente.' / 'Funds collected from fines imposed on offenders shall revert in favour of the district chamber with jurisdiction over the area where the infraction was recorded, of the agent or group of agents who imposed the fine, in the form of an emolument, as well as in favour of the Fund for the Environment referred to in the Basic Environmental Law.' Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>0.77</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
+      <c r="O16" s="2" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>0.6</v>
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
@@ -2236,25 +1942,19 @@
           <t>Art. 39.º(1): funds collected from fines imposed on offenders revert in favour of the District Chamber with jurisdiction over the area where the infraction was recorded, of the agent(s) who imposed the fine, in the form of an emolument, and in favour of the Fund for the Environment referred to in the Basic Environmental Law. Art. 39.º(2): the distribution formula for these shares shall be defined by order of the minister responsible for the environment.</t>
         </is>
       </c>
-      <c r="S16" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T16" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="S16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>0.5</v>
       </c>
       <c r="U16" s="2" t="inlineStr">
         <is>
           <t>Authority: District Chambers, enforcing agents and the National Fund for the Environment are explicitly named as beneficiaries, with the distribution formula to be set by the environment minister (+0.25). No enforcement sub-score applicable to a funding-allocation rule (0). No monitoring mechanism specified (0). Unconditional: no exemptions are stated to the allocation rule itself (+0.25).</t>
         </is>
       </c>
-      <c r="V16" s="2" t="inlineStr">
-        <is>
-          <t>0.55</t>
-        </is>
+      <c r="V16" s="2" t="n">
+        <v>0.55</v>
       </c>
       <c r="W16" s="2" t="inlineStr">
         <is>

</xml_diff>